<commit_message>
record the new groups path in the cluster design manifests
</commit_message>
<xml_diff>
--- a/03_Cluster_groups/Muscle_size/02_Design_Contrasts/c_data/design_contrasts.xlsx
+++ b/03_Cluster_groups/Muscle_size/02_Design_Contrasts/c_data/design_contrasts.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="182">
   <si>
     <t>sheet</t>
   </si>
@@ -210,7 +210,7 @@
     <t>groups</t>
   </si>
   <si>
-    <t>03_Cluster_groups/Muscle_size/01_Clustering/c_data/groups.rds</t>
+    <t>02_Groups/Muscle_size/c_data/groups.rds</t>
   </si>
   <si>
     <t>e05c84ed32b4787b0edbe8e6a90130ad</t>
@@ -559,6 +559,12 @@
   </si>
   <si>
     <t>1.7.1</t>
+  </si>
+  <si>
+    <t>yaml</t>
+  </si>
+  <si>
+    <t>2.3.12</t>
   </si>
 </sst>
 </file>
@@ -1290,7 +1296,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -1931,6 +1937,17 @@
         <v>70</v>
       </c>
     </row>
+    <row r="59" spans="1:3">
+      <c r="A59" t="s">
+        <v>180</v>
+      </c>
+      <c r="B59" t="s">
+        <v>181</v>
+      </c>
+      <c r="C59" t="s">
+        <v>70</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>